<commit_message>
fixed wrong mapping of few regions
</commit_message>
<xml_diff>
--- a/datasets/Penyesuaian_IndoGeospasial.xlsx
+++ b/datasets/Penyesuaian_IndoGeospasial.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python-stuff\UAS_ML\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBEB38B4-9745-45E6-BE51-89197D4D3C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB13D9A9-0E6F-4172-9E7B-A209D7399E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5700" yWindow="2340" windowWidth="17280" windowHeight="9180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="1028">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="1028">
   <si>
     <t>Aceh Barat</t>
   </si>
@@ -2328,9 +2328,6 @@
     <t>Pangkajene dan Kepulauan</t>
   </si>
   <si>
-    <t>PANGANDARAN</t>
-  </si>
-  <si>
     <t>Paniai</t>
   </si>
   <si>
@@ -3109,6 +3106,9 @@
   </si>
   <si>
     <t>YALIMO</t>
+  </si>
+  <si>
+    <t>POHUWATO</t>
   </si>
 </sst>
 </file>
@@ -3426,7 +3426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B514"/>
+  <dimension ref="A1:B515"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.77734375" customWidth="1"/>
@@ -6503,1047 +6503,1052 @@
         <v>766</v>
       </c>
       <c r="B384" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
     </row>
     <row r="385" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B385" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
     </row>
     <row r="386" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="B386" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
     </row>
     <row r="387" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B387" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
     </row>
     <row r="388" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B388" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
     </row>
     <row r="389" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B389" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
     </row>
     <row r="390" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B390" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
     </row>
     <row r="391" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B391" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
     </row>
     <row r="392" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B392" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
     </row>
     <row r="393" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="B393" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
     </row>
     <row r="394" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B394" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
     </row>
     <row r="395" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B395" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
     </row>
     <row r="396" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B396" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
     </row>
     <row r="397" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B397" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
     </row>
     <row r="398" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B398" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
     </row>
     <row r="399" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B399" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
     </row>
     <row r="400" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B400" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
     </row>
     <row r="401" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B401" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
     </row>
     <row r="402" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B402" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
     </row>
     <row r="403" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B403" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
     </row>
     <row r="404" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B404" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
     </row>
     <row r="405" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B405" t="s">
-        <v>809</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="406" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
+        <v>809</v>
+      </c>
+      <c r="B406" t="s">
         <v>810</v>
-      </c>
-      <c r="B406" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="407" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
+        <v>811</v>
+      </c>
+      <c r="B407" t="s">
         <v>812</v>
-      </c>
-      <c r="B407" t="s">
-        <v>813</v>
       </c>
     </row>
     <row r="408" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
+        <v>813</v>
+      </c>
+      <c r="B408" t="s">
         <v>814</v>
-      </c>
-      <c r="B408" t="s">
-        <v>815</v>
       </c>
     </row>
     <row r="409" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
+        <v>815</v>
+      </c>
+      <c r="B409" t="s">
         <v>816</v>
-      </c>
-      <c r="B409" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="410" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
+        <v>817</v>
+      </c>
+      <c r="B410" t="s">
         <v>818</v>
-      </c>
-      <c r="B410" t="s">
-        <v>819</v>
       </c>
     </row>
     <row r="411" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A411" t="s">
+        <v>819</v>
+      </c>
+      <c r="B411" t="s">
         <v>820</v>
-      </c>
-      <c r="B411" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="412" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
+        <v>821</v>
+      </c>
+      <c r="B412" t="s">
         <v>822</v>
-      </c>
-      <c r="B412" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="413" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
+        <v>823</v>
+      </c>
+      <c r="B413" t="s">
         <v>824</v>
-      </c>
-      <c r="B413" t="s">
-        <v>825</v>
       </c>
     </row>
     <row r="414" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
+        <v>825</v>
+      </c>
+      <c r="B414" t="s">
         <v>826</v>
-      </c>
-      <c r="B414" t="s">
-        <v>827</v>
       </c>
     </row>
     <row r="415" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
+        <v>827</v>
+      </c>
+      <c r="B415" t="s">
         <v>828</v>
-      </c>
-      <c r="B415" t="s">
-        <v>829</v>
       </c>
     </row>
     <row r="416" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
+        <v>829</v>
+      </c>
+      <c r="B416" t="s">
         <v>830</v>
-      </c>
-      <c r="B416" t="s">
-        <v>831</v>
       </c>
     </row>
     <row r="417" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
+        <v>831</v>
+      </c>
+      <c r="B417" t="s">
         <v>832</v>
-      </c>
-      <c r="B417" t="s">
-        <v>833</v>
       </c>
     </row>
     <row r="418" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
+        <v>833</v>
+      </c>
+      <c r="B418" t="s">
         <v>834</v>
-      </c>
-      <c r="B418" t="s">
-        <v>835</v>
       </c>
     </row>
     <row r="419" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
+        <v>835</v>
+      </c>
+      <c r="B419" t="s">
         <v>836</v>
-      </c>
-      <c r="B419" t="s">
-        <v>837</v>
       </c>
     </row>
     <row r="420" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
+        <v>837</v>
+      </c>
+      <c r="B420" t="s">
         <v>838</v>
-      </c>
-      <c r="B420" t="s">
-        <v>839</v>
       </c>
     </row>
     <row r="421" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
+        <v>839</v>
+      </c>
+      <c r="B421" t="s">
         <v>840</v>
-      </c>
-      <c r="B421" t="s">
-        <v>841</v>
       </c>
     </row>
     <row r="422" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
+        <v>841</v>
+      </c>
+      <c r="B422" t="s">
         <v>842</v>
-      </c>
-      <c r="B422" t="s">
-        <v>843</v>
       </c>
     </row>
     <row r="423" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
+        <v>843</v>
+      </c>
+      <c r="B423" t="s">
         <v>844</v>
-      </c>
-      <c r="B423" t="s">
-        <v>845</v>
       </c>
     </row>
     <row r="424" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
+        <v>845</v>
+      </c>
+      <c r="B424" t="s">
         <v>846</v>
-      </c>
-      <c r="B424" t="s">
-        <v>847</v>
       </c>
     </row>
     <row r="425" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
+        <v>847</v>
+      </c>
+      <c r="B425" t="s">
         <v>848</v>
-      </c>
-      <c r="B425" t="s">
-        <v>849</v>
       </c>
     </row>
     <row r="426" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
+        <v>849</v>
+      </c>
+      <c r="B426" t="s">
         <v>850</v>
-      </c>
-      <c r="B426" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="427" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
+        <v>851</v>
+      </c>
+      <c r="B427" t="s">
         <v>852</v>
-      </c>
-      <c r="B427" t="s">
-        <v>853</v>
       </c>
     </row>
     <row r="428" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
+        <v>853</v>
+      </c>
+      <c r="B428" t="s">
         <v>854</v>
-      </c>
-      <c r="B428" t="s">
-        <v>855</v>
       </c>
     </row>
     <row r="429" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
+        <v>855</v>
+      </c>
+      <c r="B429" t="s">
         <v>856</v>
-      </c>
-      <c r="B429" t="s">
-        <v>857</v>
       </c>
     </row>
     <row r="430" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
+        <v>857</v>
+      </c>
+      <c r="B430" t="s">
         <v>858</v>
-      </c>
-      <c r="B430" t="s">
-        <v>859</v>
       </c>
     </row>
     <row r="431" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
+        <v>859</v>
+      </c>
+      <c r="B431" t="s">
         <v>860</v>
-      </c>
-      <c r="B431" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="432" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
+        <v>861</v>
+      </c>
+      <c r="B432" t="s">
         <v>862</v>
-      </c>
-      <c r="B432" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="433" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
+        <v>863</v>
+      </c>
+      <c r="B433" t="s">
         <v>864</v>
-      </c>
-      <c r="B433" t="s">
-        <v>865</v>
       </c>
     </row>
     <row r="434" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A434" t="s">
+        <v>865</v>
+      </c>
+      <c r="B434" t="s">
         <v>866</v>
-      </c>
-      <c r="B434" t="s">
-        <v>867</v>
       </c>
     </row>
     <row r="435" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
+        <v>867</v>
+      </c>
+      <c r="B435" t="s">
         <v>868</v>
-      </c>
-      <c r="B435" t="s">
-        <v>869</v>
       </c>
     </row>
     <row r="436" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
+        <v>869</v>
+      </c>
+      <c r="B436" t="s">
         <v>870</v>
-      </c>
-      <c r="B436" t="s">
-        <v>871</v>
       </c>
     </row>
     <row r="437" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
+        <v>871</v>
+      </c>
+      <c r="B437" t="s">
         <v>872</v>
-      </c>
-      <c r="B437" t="s">
-        <v>873</v>
       </c>
     </row>
     <row r="438" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
+        <v>873</v>
+      </c>
+      <c r="B438" t="s">
         <v>874</v>
-      </c>
-      <c r="B438" t="s">
-        <v>875</v>
       </c>
     </row>
     <row r="439" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
+        <v>875</v>
+      </c>
+      <c r="B439" t="s">
         <v>876</v>
-      </c>
-      <c r="B439" t="s">
-        <v>877</v>
       </c>
     </row>
     <row r="440" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A440" t="s">
+        <v>877</v>
+      </c>
+      <c r="B440" t="s">
         <v>878</v>
-      </c>
-      <c r="B440" t="s">
-        <v>879</v>
       </c>
     </row>
     <row r="441" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A441" t="s">
+        <v>879</v>
+      </c>
+      <c r="B441" t="s">
         <v>880</v>
-      </c>
-      <c r="B441" t="s">
-        <v>881</v>
       </c>
     </row>
     <row r="442" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
+        <v>881</v>
+      </c>
+      <c r="B442" t="s">
         <v>882</v>
-      </c>
-      <c r="B442" t="s">
-        <v>883</v>
       </c>
     </row>
     <row r="443" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
+        <v>883</v>
+      </c>
+      <c r="B443" t="s">
         <v>884</v>
-      </c>
-      <c r="B443" t="s">
-        <v>885</v>
       </c>
     </row>
     <row r="444" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
+        <v>885</v>
+      </c>
+      <c r="B444" t="s">
         <v>886</v>
-      </c>
-      <c r="B444" t="s">
-        <v>887</v>
       </c>
     </row>
     <row r="445" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
+        <v>887</v>
+      </c>
+      <c r="B445" t="s">
         <v>888</v>
-      </c>
-      <c r="B445" t="s">
-        <v>889</v>
       </c>
     </row>
     <row r="446" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
+        <v>889</v>
+      </c>
+      <c r="B446" t="s">
         <v>890</v>
-      </c>
-      <c r="B446" t="s">
-        <v>891</v>
       </c>
     </row>
     <row r="447" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
+        <v>891</v>
+      </c>
+      <c r="B447" t="s">
         <v>892</v>
-      </c>
-      <c r="B447" t="s">
-        <v>893</v>
       </c>
     </row>
     <row r="448" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
+        <v>893</v>
+      </c>
+      <c r="B448" t="s">
         <v>894</v>
-      </c>
-      <c r="B448" t="s">
-        <v>895</v>
       </c>
     </row>
     <row r="449" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
+        <v>895</v>
+      </c>
+      <c r="B449" t="s">
         <v>896</v>
-      </c>
-      <c r="B449" t="s">
-        <v>897</v>
       </c>
     </row>
     <row r="450" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
+        <v>897</v>
+      </c>
+      <c r="B450" t="s">
         <v>898</v>
-      </c>
-      <c r="B450" t="s">
-        <v>899</v>
       </c>
     </row>
     <row r="451" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A451" t="s">
+        <v>899</v>
+      </c>
+      <c r="B451" t="s">
         <v>900</v>
-      </c>
-      <c r="B451" t="s">
-        <v>901</v>
       </c>
     </row>
     <row r="452" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
+        <v>901</v>
+      </c>
+      <c r="B452" t="s">
         <v>902</v>
-      </c>
-      <c r="B452" t="s">
-        <v>903</v>
       </c>
     </row>
     <row r="453" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
+        <v>903</v>
+      </c>
+      <c r="B453" t="s">
         <v>904</v>
-      </c>
-      <c r="B453" t="s">
-        <v>905</v>
       </c>
     </row>
     <row r="454" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A454" t="s">
+        <v>905</v>
+      </c>
+      <c r="B454" t="s">
         <v>906</v>
-      </c>
-      <c r="B454" t="s">
-        <v>907</v>
       </c>
     </row>
     <row r="455" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
+        <v>907</v>
+      </c>
+      <c r="B455" t="s">
         <v>908</v>
-      </c>
-      <c r="B455" t="s">
-        <v>909</v>
       </c>
     </row>
     <row r="456" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
+        <v>909</v>
+      </c>
+      <c r="B456" t="s">
         <v>910</v>
-      </c>
-      <c r="B456" t="s">
-        <v>911</v>
       </c>
     </row>
     <row r="457" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A457" t="s">
+        <v>911</v>
+      </c>
+      <c r="B457" t="s">
         <v>912</v>
-      </c>
-      <c r="B457" t="s">
-        <v>913</v>
       </c>
     </row>
     <row r="458" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A458" t="s">
+        <v>913</v>
+      </c>
+      <c r="B458" t="s">
         <v>914</v>
-      </c>
-      <c r="B458" t="s">
-        <v>915</v>
       </c>
     </row>
     <row r="459" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A459" t="s">
+        <v>915</v>
+      </c>
+      <c r="B459" t="s">
         <v>916</v>
-      </c>
-      <c r="B459" t="s">
-        <v>917</v>
       </c>
     </row>
     <row r="460" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A460" t="s">
+        <v>917</v>
+      </c>
+      <c r="B460" t="s">
         <v>918</v>
-      </c>
-      <c r="B460" t="s">
-        <v>919</v>
       </c>
     </row>
     <row r="461" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A461" t="s">
+        <v>919</v>
+      </c>
+      <c r="B461" t="s">
         <v>920</v>
-      </c>
-      <c r="B461" t="s">
-        <v>921</v>
       </c>
     </row>
     <row r="462" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A462" t="s">
+        <v>921</v>
+      </c>
+      <c r="B462" t="s">
         <v>922</v>
-      </c>
-      <c r="B462" t="s">
-        <v>923</v>
       </c>
     </row>
     <row r="463" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A463" t="s">
+        <v>923</v>
+      </c>
+      <c r="B463" t="s">
         <v>924</v>
-      </c>
-      <c r="B463" t="s">
-        <v>925</v>
       </c>
     </row>
     <row r="464" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A464" t="s">
+        <v>925</v>
+      </c>
+      <c r="B464" t="s">
         <v>926</v>
-      </c>
-      <c r="B464" t="s">
-        <v>927</v>
       </c>
     </row>
     <row r="465" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A465" t="s">
+        <v>927</v>
+      </c>
+      <c r="B465" t="s">
         <v>928</v>
-      </c>
-      <c r="B465" t="s">
-        <v>929</v>
       </c>
     </row>
     <row r="466" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A466" t="s">
+        <v>929</v>
+      </c>
+      <c r="B466" t="s">
         <v>930</v>
-      </c>
-      <c r="B466" t="s">
-        <v>931</v>
       </c>
     </row>
     <row r="467" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A467" t="s">
+        <v>931</v>
+      </c>
+      <c r="B467" t="s">
         <v>932</v>
-      </c>
-      <c r="B467" t="s">
-        <v>933</v>
       </c>
     </row>
     <row r="468" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A468" t="s">
+        <v>933</v>
+      </c>
+      <c r="B468" t="s">
         <v>934</v>
-      </c>
-      <c r="B468" t="s">
-        <v>935</v>
       </c>
     </row>
     <row r="469" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A469" t="s">
+        <v>935</v>
+      </c>
+      <c r="B469" t="s">
         <v>936</v>
-      </c>
-      <c r="B469" t="s">
-        <v>937</v>
       </c>
     </row>
     <row r="470" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A470" t="s">
+        <v>937</v>
+      </c>
+      <c r="B470" t="s">
         <v>938</v>
-      </c>
-      <c r="B470" t="s">
-        <v>939</v>
       </c>
     </row>
     <row r="471" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A471" t="s">
+        <v>939</v>
+      </c>
+      <c r="B471" t="s">
         <v>940</v>
-      </c>
-      <c r="B471" t="s">
-        <v>941</v>
       </c>
     </row>
     <row r="472" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A472" t="s">
+        <v>941</v>
+      </c>
+      <c r="B472" t="s">
         <v>942</v>
-      </c>
-      <c r="B472" t="s">
-        <v>943</v>
       </c>
     </row>
     <row r="473" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A473" t="s">
+        <v>943</v>
+      </c>
+      <c r="B473" t="s">
         <v>944</v>
-      </c>
-      <c r="B473" t="s">
-        <v>945</v>
       </c>
     </row>
     <row r="474" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A474" t="s">
+        <v>945</v>
+      </c>
+      <c r="B474" t="s">
         <v>946</v>
-      </c>
-      <c r="B474" t="s">
-        <v>947</v>
       </c>
     </row>
     <row r="475" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A475" t="s">
+        <v>947</v>
+      </c>
+      <c r="B475" t="s">
         <v>948</v>
-      </c>
-      <c r="B475" t="s">
-        <v>949</v>
       </c>
     </row>
     <row r="476" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A476" t="s">
+        <v>949</v>
+      </c>
+      <c r="B476" t="s">
         <v>950</v>
-      </c>
-      <c r="B476" t="s">
-        <v>951</v>
       </c>
     </row>
     <row r="477" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A477" t="s">
+        <v>951</v>
+      </c>
+      <c r="B477" t="s">
         <v>952</v>
-      </c>
-      <c r="B477" t="s">
-        <v>953</v>
       </c>
     </row>
     <row r="478" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A478" t="s">
+        <v>953</v>
+      </c>
+      <c r="B478" t="s">
         <v>954</v>
-      </c>
-      <c r="B478" t="s">
-        <v>955</v>
       </c>
     </row>
     <row r="479" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A479" t="s">
+        <v>955</v>
+      </c>
+      <c r="B479" t="s">
         <v>956</v>
-      </c>
-      <c r="B479" t="s">
-        <v>957</v>
       </c>
     </row>
     <row r="480" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A480" t="s">
+        <v>957</v>
+      </c>
+      <c r="B480" t="s">
         <v>958</v>
-      </c>
-      <c r="B480" t="s">
-        <v>959</v>
       </c>
     </row>
     <row r="481" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A481" t="s">
+        <v>959</v>
+      </c>
+      <c r="B481" t="s">
         <v>960</v>
-      </c>
-      <c r="B481" t="s">
-        <v>961</v>
       </c>
     </row>
     <row r="482" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A482" t="s">
+        <v>961</v>
+      </c>
+      <c r="B482" t="s">
         <v>962</v>
-      </c>
-      <c r="B482" t="s">
-        <v>963</v>
       </c>
     </row>
     <row r="483" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A483" t="s">
+        <v>963</v>
+      </c>
+      <c r="B483" t="s">
         <v>964</v>
-      </c>
-      <c r="B483" t="s">
-        <v>965</v>
       </c>
     </row>
     <row r="484" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A484" t="s">
+        <v>965</v>
+      </c>
+      <c r="B484" t="s">
         <v>966</v>
-      </c>
-      <c r="B484" t="s">
-        <v>967</v>
       </c>
     </row>
     <row r="485" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A485" t="s">
+        <v>967</v>
+      </c>
+      <c r="B485" t="s">
         <v>968</v>
-      </c>
-      <c r="B485" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="486" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A486" t="s">
+        <v>969</v>
+      </c>
+      <c r="B486" t="s">
         <v>970</v>
-      </c>
-      <c r="B486" t="s">
-        <v>971</v>
       </c>
     </row>
     <row r="487" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A487" t="s">
+        <v>971</v>
+      </c>
+      <c r="B487" t="s">
         <v>972</v>
-      </c>
-      <c r="B487" t="s">
-        <v>973</v>
       </c>
     </row>
     <row r="488" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A488" t="s">
+        <v>973</v>
+      </c>
+      <c r="B488" t="s">
         <v>974</v>
-      </c>
-      <c r="B488" t="s">
-        <v>975</v>
       </c>
     </row>
     <row r="489" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A489" t="s">
+        <v>975</v>
+      </c>
+      <c r="B489" t="s">
         <v>976</v>
-      </c>
-      <c r="B489" t="s">
-        <v>977</v>
       </c>
     </row>
     <row r="490" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A490" t="s">
+        <v>977</v>
+      </c>
+      <c r="B490" t="s">
         <v>978</v>
-      </c>
-      <c r="B490" t="s">
-        <v>979</v>
       </c>
     </row>
     <row r="491" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A491" t="s">
+        <v>979</v>
+      </c>
+      <c r="B491" t="s">
         <v>980</v>
-      </c>
-      <c r="B491" t="s">
-        <v>981</v>
       </c>
     </row>
     <row r="492" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A492" t="s">
+        <v>981</v>
+      </c>
+      <c r="B492" t="s">
         <v>982</v>
-      </c>
-      <c r="B492" t="s">
-        <v>983</v>
       </c>
     </row>
     <row r="493" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A493" t="s">
+        <v>983</v>
+      </c>
+      <c r="B493" t="s">
         <v>984</v>
-      </c>
-      <c r="B493" t="s">
-        <v>985</v>
       </c>
     </row>
     <row r="494" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A494" t="s">
+        <v>985</v>
+      </c>
+      <c r="B494" t="s">
         <v>986</v>
-      </c>
-      <c r="B494" t="s">
-        <v>987</v>
       </c>
     </row>
     <row r="495" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A495" t="s">
+        <v>987</v>
+      </c>
+      <c r="B495" t="s">
         <v>988</v>
-      </c>
-      <c r="B495" t="s">
-        <v>989</v>
       </c>
     </row>
     <row r="496" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A496" t="s">
+        <v>989</v>
+      </c>
+      <c r="B496" t="s">
         <v>990</v>
-      </c>
-      <c r="B496" t="s">
-        <v>991</v>
       </c>
     </row>
     <row r="497" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A497" t="s">
+        <v>991</v>
+      </c>
+      <c r="B497" t="s">
         <v>992</v>
-      </c>
-      <c r="B497" t="s">
-        <v>993</v>
       </c>
     </row>
     <row r="498" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A498" t="s">
+        <v>993</v>
+      </c>
+      <c r="B498" t="s">
         <v>994</v>
-      </c>
-      <c r="B498" t="s">
-        <v>995</v>
       </c>
     </row>
     <row r="499" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A499" t="s">
+        <v>995</v>
+      </c>
+      <c r="B499" t="s">
         <v>996</v>
-      </c>
-      <c r="B499" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="500" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A500" t="s">
+        <v>997</v>
+      </c>
+      <c r="B500" t="s">
         <v>998</v>
-      </c>
-      <c r="B500" t="s">
-        <v>999</v>
       </c>
     </row>
     <row r="501" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A501" t="s">
+        <v>999</v>
+      </c>
+      <c r="B501" t="s">
         <v>1000</v>
-      </c>
-      <c r="B501" t="s">
-        <v>1001</v>
       </c>
     </row>
     <row r="502" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A502" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B502" t="s">
         <v>1002</v>
-      </c>
-      <c r="B502" t="s">
-        <v>1003</v>
       </c>
     </row>
     <row r="503" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A503" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B503" t="s">
         <v>1004</v>
-      </c>
-      <c r="B503" t="s">
-        <v>1005</v>
       </c>
     </row>
     <row r="504" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A504" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B504" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="505" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A505" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B505" t="s">
-        <v>1009</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="506" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A506" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B506" t="s">
         <v>1010</v>
-      </c>
-      <c r="B506" t="s">
-        <v>1011</v>
       </c>
     </row>
     <row r="507" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A507" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B507" t="s">
         <v>1012</v>
-      </c>
-      <c r="B507" t="s">
-        <v>1013</v>
       </c>
     </row>
     <row r="508" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A508" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B508" t="s">
         <v>1014</v>
-      </c>
-      <c r="B508" t="s">
-        <v>1015</v>
       </c>
     </row>
     <row r="509" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A509" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B509" t="s">
         <v>1016</v>
-      </c>
-      <c r="B509" t="s">
-        <v>1017</v>
       </c>
     </row>
     <row r="510" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A510" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B510" t="s">
         <v>1018</v>
-      </c>
-      <c r="B510" t="s">
-        <v>1019</v>
       </c>
     </row>
     <row r="511" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A511" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B511" t="s">
         <v>1020</v>
-      </c>
-      <c r="B511" t="s">
-        <v>1021</v>
       </c>
     </row>
     <row r="512" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A512" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B512" t="s">
         <v>1022</v>
-      </c>
-      <c r="B512" t="s">
-        <v>1023</v>
       </c>
     </row>
     <row r="513" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A513" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B513" t="s">
         <v>1024</v>
-      </c>
-      <c r="B513" t="s">
-        <v>1025</v>
       </c>
     </row>
     <row r="514" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A514" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B514" t="s">
         <v>1026</v>
       </c>
-      <c r="B514" t="s">
-        <v>1027</v>
+    </row>
+    <row r="515" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B515" t="s">
+        <v>1026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>